<commit_message>
Fix video publish schedule 4-day gap, analytics graph alignment and CRM publish date modulation
</commit_message>
<xml_diff>
--- a/YouTube_Studio_CMS_Template_Kids_Content.xlsx
+++ b/YouTube_Studio_CMS_Template_Kids_Content.xlsx
@@ -670,7 +670,7 @@
         <v>https://youtu.be/demo1</v>
       </c>
       <c r="F2" t="str">
-        <v>2026-07-17</v>
+        <v>2026-08-16</v>
       </c>
       <c r="G2" t="str">
         <v>Public</v>
@@ -738,7 +738,7 @@
         <v>https://youtu.be/demo2</v>
       </c>
       <c r="F3" t="str">
-        <v>2026-04-16</v>
+        <v>2026-08-12</v>
       </c>
       <c r="G3" t="str">
         <v>Public</v>
@@ -806,7 +806,7 @@
         <v>https://youtu.be/demo3</v>
       </c>
       <c r="F4" t="str">
-        <v>2026-04-27</v>
+        <v>2026-08-08</v>
       </c>
       <c r="G4" t="str">
         <v>Public</v>
@@ -874,7 +874,7 @@
         <v>https://youtu.be/demo4</v>
       </c>
       <c r="F5" t="str">
-        <v>2026-05-08</v>
+        <v>2026-08-04</v>
       </c>
       <c r="G5" t="str">
         <v>Public</v>
@@ -942,7 +942,7 @@
         <v>https://youtu.be/demo5</v>
       </c>
       <c r="F6" t="str">
-        <v>2026-05-19</v>
+        <v>2026-07-31</v>
       </c>
       <c r="G6" t="str">
         <v>Public</v>
@@ -1010,7 +1010,7 @@
         <v>https://youtu.be/demo6</v>
       </c>
       <c r="F7" t="str">
-        <v>2026-05-30</v>
+        <v>2026-07-27</v>
       </c>
       <c r="G7" t="str">
         <v>Public</v>
@@ -1078,7 +1078,7 @@
         <v>https://youtu.be/demo7</v>
       </c>
       <c r="F8" t="str">
-        <v>2026-06-10</v>
+        <v>2026-07-23</v>
       </c>
       <c r="G8" t="str">
         <v>Public</v>
@@ -1146,7 +1146,7 @@
         <v>https://youtu.be/demo8</v>
       </c>
       <c r="F9" t="str">
-        <v>2026-06-21</v>
+        <v>2026-07-19</v>
       </c>
       <c r="G9" t="str">
         <v>Public</v>
@@ -1214,7 +1214,7 @@
         <v>https://youtu.be/demo9</v>
       </c>
       <c r="F10" t="str">
-        <v>2026-07-02</v>
+        <v>2026-07-15</v>
       </c>
       <c r="G10" t="str">
         <v>Public</v>
@@ -1282,7 +1282,7 @@
         <v>https://youtu.be/demo10</v>
       </c>
       <c r="F11" t="str">
-        <v>2026-07-13</v>
+        <v>2026-07-11</v>
       </c>
       <c r="G11" t="str">
         <v>Public</v>

</xml_diff>